<commit_message>
update generated data Triggered by 05156012e78030ebdd8e3f25f9ba18a1fd33f3f6
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F332"/>
+  <dimension ref="A1:F333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9095,44 +9095,44 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -9159,12 +9159,12 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
@@ -9191,12 +9191,12 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -9206,7 +9206,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -9223,12 +9223,12 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9238,7 +9238,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -9255,12 +9255,12 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -9287,12 +9287,12 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9319,12 +9319,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9351,12 +9351,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9366,29 +9366,29 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9398,29 +9398,29 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9430,7 +9430,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9447,12 +9447,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9479,12 +9479,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9494,7 +9494,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9511,12 +9511,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9543,12 +9543,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9575,12 +9575,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9607,12 +9607,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9622,7 +9622,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9639,12 +9639,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9654,29 +9654,29 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9686,29 +9686,29 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9718,29 +9718,29 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9750,7 +9750,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9767,12 +9767,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9782,7 +9782,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9799,12 +9799,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9831,12 +9831,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9863,12 +9863,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9878,29 +9878,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9910,29 +9910,29 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9942,7 +9942,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9959,12 +9959,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9974,7 +9974,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9991,12 +9991,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -10006,29 +10006,29 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10038,29 +10038,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10070,7 +10070,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10087,12 +10087,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10102,29 +10102,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10134,29 +10134,29 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10183,12 +10183,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10198,7 +10198,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -10215,12 +10215,12 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10247,12 +10247,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10294,29 +10294,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10326,29 +10326,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10358,7 +10358,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10375,12 +10375,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10407,12 +10407,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10439,12 +10439,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10454,29 +10454,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10486,29 +10486,29 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10535,12 +10535,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10550,7 +10550,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10567,12 +10567,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10599,12 +10599,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10631,12 +10631,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10646,7 +10646,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10663,12 +10663,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10695,12 +10695,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10710,29 +10710,29 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10742,29 +10742,29 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10791,12 +10791,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10806,7 +10806,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10823,12 +10823,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10838,7 +10838,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10855,12 +10855,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10870,7 +10870,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10887,12 +10887,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10902,29 +10902,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10951,30 +10951,62 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
+      <c r="B333" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C332" t="inlineStr">
+      <c r="C333" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D332" t="inlineStr">
+      <c r="D333" t="inlineStr">
         <is>
           <t>Winnipeg, MB</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr">
+      <c r="E333" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr">
+      <c r="F333" t="inlineStr">
         <is>
           <t>CA</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 78f9f6b4b1ef845ce83fed596e96d261383d8252
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F334"/>
+  <dimension ref="A1:F335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9159,44 +9159,44 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -9206,7 +9206,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -9223,12 +9223,12 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9238,7 +9238,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -9255,12 +9255,12 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -9287,12 +9287,12 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9319,12 +9319,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9351,12 +9351,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9383,12 +9383,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9415,12 +9415,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9430,29 +9430,29 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9462,29 +9462,29 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9494,7 +9494,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9511,12 +9511,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9543,12 +9543,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9575,12 +9575,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9607,12 +9607,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9622,7 +9622,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9639,12 +9639,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9654,7 +9654,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9671,12 +9671,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9703,12 +9703,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9718,29 +9718,29 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9750,29 +9750,29 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9782,29 +9782,29 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9831,12 +9831,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9863,12 +9863,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9895,12 +9895,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9927,12 +9927,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9942,29 +9942,29 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9974,29 +9974,29 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -10006,7 +10006,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10023,12 +10023,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10055,12 +10055,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10070,29 +10070,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10102,29 +10102,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10134,7 +10134,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10151,12 +10151,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10166,29 +10166,29 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10198,29 +10198,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10247,12 +10247,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10294,7 +10294,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10311,12 +10311,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10343,12 +10343,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10358,29 +10358,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10390,29 +10390,29 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10439,12 +10439,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10454,7 +10454,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10471,12 +10471,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10486,7 +10486,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10503,12 +10503,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10518,29 +10518,29 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10550,29 +10550,29 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10599,12 +10599,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10631,12 +10631,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10646,7 +10646,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10663,12 +10663,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10695,12 +10695,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10727,12 +10727,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10742,7 +10742,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10759,12 +10759,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10774,29 +10774,29 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10806,29 +10806,29 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10838,7 +10838,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10855,12 +10855,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10870,7 +10870,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10887,12 +10887,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10919,12 +10919,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10951,12 +10951,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10966,29 +10966,29 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11015,30 +11015,62 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B334" t="inlineStr">
+      <c r="B335" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C334" t="inlineStr">
+      <c r="C335" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr">
+      <c r="D335" t="inlineStr">
         <is>
           <t>Winnipeg, MB</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr">
+      <c r="E335" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr">
+      <c r="F335" t="inlineStr">
         <is>
           <t>CA</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 51848c467b645e8523c77f34d6d6921734c1bbb8
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F335"/>
+  <dimension ref="A1:F336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9191,44 +9191,44 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9238,7 +9238,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -9255,12 +9255,12 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -9287,12 +9287,12 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9319,12 +9319,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9351,12 +9351,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9383,12 +9383,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9415,12 +9415,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9430,7 +9430,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9447,12 +9447,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9462,29 +9462,29 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9494,29 +9494,29 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9543,12 +9543,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9575,12 +9575,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9607,12 +9607,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9622,7 +9622,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9639,12 +9639,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9654,7 +9654,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9671,12 +9671,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9703,12 +9703,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9735,12 +9735,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9750,29 +9750,29 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9782,29 +9782,29 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9814,29 +9814,29 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9863,12 +9863,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9895,12 +9895,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9927,12 +9927,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9942,7 +9942,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9959,12 +9959,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9974,29 +9974,29 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -10006,29 +10006,29 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10055,12 +10055,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10070,7 +10070,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10087,12 +10087,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10102,29 +10102,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10134,29 +10134,29 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10183,12 +10183,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10198,29 +10198,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10230,29 +10230,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10294,7 +10294,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10311,12 +10311,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10343,12 +10343,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10358,7 +10358,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10375,12 +10375,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10390,29 +10390,29 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10422,29 +10422,29 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10454,7 +10454,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10471,12 +10471,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10486,7 +10486,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10503,12 +10503,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10535,12 +10535,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10550,29 +10550,29 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10582,29 +10582,29 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10631,12 +10631,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10646,7 +10646,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10663,12 +10663,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10695,12 +10695,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10727,12 +10727,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10742,7 +10742,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10759,12 +10759,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10791,12 +10791,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10806,29 +10806,29 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10838,29 +10838,29 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10870,7 +10870,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10887,12 +10887,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10919,12 +10919,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10951,12 +10951,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10966,7 +10966,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10983,12 +10983,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10998,29 +10998,29 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11030,7 +11030,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11047,30 +11047,62 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr">
+      <c r="B336" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C335" t="inlineStr">
+      <c r="C336" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr">
+      <c r="D336" t="inlineStr">
         <is>
           <t>Winnipeg, MB</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr">
+      <c r="E336" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr">
+      <c r="F336" t="inlineStr">
         <is>
           <t>CA</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by b0166ccc1dabd602d88824178c761493d82bc104
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F337"/>
+  <dimension ref="A1:F338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9255,44 +9255,44 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9319,12 +9319,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9351,12 +9351,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9383,12 +9383,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9415,12 +9415,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9430,7 +9430,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9447,12 +9447,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9479,12 +9479,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9494,7 +9494,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9511,12 +9511,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9526,29 +9526,29 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9558,29 +9558,29 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9607,12 +9607,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9622,7 +9622,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9639,12 +9639,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9654,7 +9654,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9671,12 +9671,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9703,12 +9703,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9735,12 +9735,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9750,7 +9750,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9767,12 +9767,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9782,7 +9782,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9799,12 +9799,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9814,29 +9814,29 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9846,29 +9846,29 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9878,29 +9878,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9927,12 +9927,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9942,7 +9942,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9959,12 +9959,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9974,7 +9974,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9991,12 +9991,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -10006,7 +10006,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10023,12 +10023,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10038,29 +10038,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10070,29 +10070,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10102,7 +10102,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10119,12 +10119,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10134,7 +10134,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10151,12 +10151,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10166,29 +10166,29 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10198,29 +10198,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10247,12 +10247,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10262,29 +10262,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10294,29 +10294,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10343,12 +10343,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10358,7 +10358,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10375,12 +10375,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10407,12 +10407,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10439,12 +10439,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10454,29 +10454,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10486,29 +10486,29 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10535,12 +10535,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10550,7 +10550,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10567,12 +10567,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10599,12 +10599,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10614,29 +10614,29 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10646,29 +10646,29 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10695,12 +10695,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10727,12 +10727,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10742,7 +10742,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10759,12 +10759,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10791,12 +10791,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10806,7 +10806,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10823,12 +10823,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10838,7 +10838,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10855,12 +10855,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10870,29 +10870,29 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10902,29 +10902,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10951,12 +10951,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10966,7 +10966,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10983,12 +10983,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11015,12 +11015,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11030,7 +11030,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11047,12 +11047,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11062,29 +11062,29 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11111,30 +11111,62 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B338" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C338" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D338" t="inlineStr">
         <is>
           <t>Winnipeg, MB</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E338" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F338" t="inlineStr">
         <is>
           <t>CA</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 366c9b7f007abd9cddd27ad5cf3642fa4cb89fae
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F337"/>
+  <dimension ref="A1:F338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9255,44 +9255,44 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Sambalpur</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9319,12 +9319,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9351,12 +9351,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9383,12 +9383,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9415,12 +9415,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9430,7 +9430,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9447,12 +9447,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9479,12 +9479,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9494,7 +9494,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9511,12 +9511,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9526,29 +9526,29 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9558,29 +9558,29 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9607,12 +9607,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9622,7 +9622,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9639,12 +9639,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9654,7 +9654,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9671,12 +9671,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9703,12 +9703,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9735,12 +9735,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9750,7 +9750,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9767,12 +9767,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9782,7 +9782,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9799,12 +9799,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9814,29 +9814,29 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9846,29 +9846,29 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9878,29 +9878,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9927,12 +9927,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9942,7 +9942,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9959,12 +9959,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9974,7 +9974,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9991,12 +9991,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -10006,7 +10006,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10023,12 +10023,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10038,29 +10038,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10070,29 +10070,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10102,7 +10102,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10119,12 +10119,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10134,7 +10134,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10151,12 +10151,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10166,29 +10166,29 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10198,29 +10198,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10247,12 +10247,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10262,29 +10262,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10294,29 +10294,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10343,12 +10343,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10358,7 +10358,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10375,12 +10375,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10407,12 +10407,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10439,12 +10439,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10454,29 +10454,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10486,29 +10486,29 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10535,12 +10535,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10550,7 +10550,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10567,12 +10567,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10599,12 +10599,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10614,29 +10614,29 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10646,29 +10646,29 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10695,12 +10695,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10727,12 +10727,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10742,7 +10742,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10759,12 +10759,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10791,12 +10791,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10806,7 +10806,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10823,12 +10823,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10838,7 +10838,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10855,12 +10855,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10870,29 +10870,29 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10902,29 +10902,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10951,12 +10951,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10966,7 +10966,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10983,12 +10983,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11015,12 +11015,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11030,7 +11030,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11047,12 +11047,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11062,29 +11062,29 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11111,30 +11111,62 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B338" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C338" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D338" t="inlineStr">
         <is>
           <t>Winnipeg, MB</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E338" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F338" t="inlineStr">
         <is>
           <t>CA</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by b8efbda50619dac2cf6ddc7807a0c54319df9d9e
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -1808,7 +1808,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Valletta, Malta</t>
+          <t>Santa Venera, Malta</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Valletta</t>
+          <t>Santa Venera</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Bogota, Colombia</t>
+          <t>Bogotá, Colombia</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Bogota</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Cacador, Brazil</t>
+          <t>Caçador, Brazil</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Cacador</t>
+          <t>Caçador</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Goiania, Brazil</t>
+          <t>Goiânia, Brazil</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Goiania</t>
+          <t>Goiânia</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Neuquen, Argentina</t>
+          <t>Neuquén, Argentina</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Neuquen</t>
+          <t>Neuquén</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Timbo, Brazil</t>
+          <t>Timbó, Brazil</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Timbo</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Uberlandia, Brazil</t>
+          <t>Uberlândia, Brazil</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Uberlandia</t>
+          <t>Uberlândia</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Dar es Salaam, Tanzania</t>
+          <t>Dar Es Salaam, Tanzania</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dar Es Salaam</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -5504,7 +5504,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Djibouti, Djibouti</t>
+          <t>Djibouti City, Djibouti</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Djibouti</t>
+          <t>Djibouti City</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Chengmai, China</t>
+          <t>Haikou, China</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Chengmai</t>
+          <t>Haikou</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -6896,7 +6896,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Shijiazhuang, China</t>
+          <t>Hengshui, China</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Shijiazhuang</t>
+          <t>Hengshui</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -7076,7 +7076,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Zibo, China</t>
+          <t>Jinan, China</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Zibo</t>
+          <t>Jinan</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -7416,7 +7416,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Male, Maldives</t>
+          <t>Malé, Maldives</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Malé</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Nanchang, China</t>
+          <t>Xinyu, China</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Nanchang</t>
+          <t>Xinyu</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">

</xml_diff>

<commit_message>
update generated data Triggered by d277371dd7e3f628056d9aabd9401ddc9d1b5dcc
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F338"/>
+  <dimension ref="A1:F337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,29 +10442,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,29 +10570,29 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,29 +10602,29 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,29 +10826,29 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,29 +10858,29 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,29 +11018,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,47 +11114,15 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>Cincinnati</t>
-        </is>
-      </c>
-      <c r="E338" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F338" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 4c993284e18e292cb2cd65315db9d945ee669fc1
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F337"/>
+  <dimension ref="A1:F338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6283,44 +6283,44 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>DLA</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Ahmedabad, India</t>
+          <t>Douala, Cameroon</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Douala</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Almaty, Kazakhstan</t>
+          <t>Ahmedabad, India</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -6330,29 +6330,29 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Almaty</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>BLR</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Bangalore, India</t>
+          <t>Almaty, Kazakhstan</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -6362,29 +6362,29 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Almaty</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>BKK</t>
+          <t>BLR</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Bangkok, Thailand</t>
+          <t>Bangalore, India</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -6394,29 +6394,29 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>BWN</t>
+          <t>BKK</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan, Brunei</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -6426,29 +6426,29 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan</t>
+          <t>Bangkok</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Brunei</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>BN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>CEB</t>
+          <t>BWN</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Cebu, Philippines</t>
+          <t>Bandar Seri Begawan, Brunei</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -6458,29 +6458,29 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Cebu</t>
+          <t>Bandar Seri Begawan</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Brunei</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>BN</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>IXC</t>
+          <t>CEB</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Chandigarh, India</t>
+          <t>Cebu, Philippines</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -6490,29 +6490,29 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Cebu</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>CGD</t>
+          <t>IXC</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Changde, China</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -6522,29 +6522,29 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Changde</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>CGD</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Chennai, India</t>
+          <t>Changde, China</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -6554,29 +6554,29 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Changde</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>CGP</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Chittagong, Bangladesh</t>
+          <t>Chennai, India</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -6586,29 +6586,29 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Chittagong</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>CMB</t>
+          <t>CGP</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Colombo, Sri Lanka</t>
+          <t>Chittagong, Bangladesh</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -6618,29 +6618,29 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Colombo</t>
+          <t>Chittagong</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>BD</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>CMB</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Dhaka, Bangladesh</t>
+          <t>Colombo, Sri Lanka</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -6650,29 +6650,29 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Colombo</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>LK</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>FUO</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Foshan, China</t>
+          <t>Dhaka, Bangladesh</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -6682,29 +6682,29 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Foshan</t>
+          <t>Dhaka</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>BD</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>FUK</t>
+          <t>FUO</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Fukuoka, Japan</t>
+          <t>Foshan, China</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -6714,29 +6714,29 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Fukuoka</t>
+          <t>Foshan</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>FOC</t>
+          <t>FUK</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Fuzhou, China</t>
+          <t>Fukuoka, Japan</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -6746,29 +6746,29 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Fuzhou</t>
+          <t>Fukuoka</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>FOC</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Guangzhou, China</t>
+          <t>Fuzhou, China</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Guangzhou</t>
+          <t>Fuzhou</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -6795,12 +6795,12 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>HAK</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Haikou, China</t>
+          <t>Guangzhou, China</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Haikou</t>
+          <t>Guangzhou</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -6827,12 +6827,12 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>HAN</t>
+          <t>HAK</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Hanoi, Vietnam</t>
+          <t>Haikou, China</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -6842,29 +6842,29 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Haikou</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>SJW</t>
+          <t>HAN</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Hengshui, China</t>
+          <t>Hanoi, Vietnam</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -6874,29 +6874,29 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Hengshui</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>SGN</t>
+          <t>SJW</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City, Vietnam</t>
+          <t>Hengshui, China</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -6906,29 +6906,29 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hengshui</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SGN</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Ho Chi Minh City, Vietnam</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -6936,19 +6936,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>HYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Hyderabad, India</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -6956,31 +6968,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="F206" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
+      <c r="D206" t="inlineStr"/>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>ISB</t>
+          <t>HYD</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Islamabad, Pakistan</t>
+          <t>Hyderabad, India</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -6990,29 +6990,29 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Islamabad</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>CGK</t>
+          <t>ISB</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Jakarta, Indonesia</t>
+          <t>Islamabad, Pakistan</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -7022,29 +7022,29 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>Islamabad</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>CGK</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Jinan, China</t>
+          <t>Jakarta, Indonesia</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -7054,29 +7054,29 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Jinan</t>
+          <t>Jakarta</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>JHB</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Johor Bahru, Malaysia</t>
+          <t>Jinan, China</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -7086,29 +7086,29 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Johor Bahru</t>
+          <t>Jinan</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>KNU</t>
+          <t>JHB</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Kanpur, India</t>
+          <t>Johor Bahru, Malaysia</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -7118,29 +7118,29 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Kanpur</t>
+          <t>Johor Bahru</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>KHH</t>
+          <t>KNU</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Kaohsiung City</t>
+          <t>Kanpur, India</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -7148,19 +7148,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D212" t="inlineStr"/>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>KHI</t>
+          <t>KHH</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Karachi, Pakistan</t>
+          <t>Kaohsiung City</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -7168,31 +7180,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr">
-        <is>
-          <t>Pakistan</t>
-        </is>
-      </c>
-      <c r="F213" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>KTM</t>
+          <t>KHI</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Kathmandu, Nepal</t>
+          <t>Karachi, Pakistan</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -7202,29 +7202,29 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Kathmandu</t>
+          <t>Karachi</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>NP</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>CCU</t>
+          <t>KTM</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Kolkata, India</t>
+          <t>Kathmandu, Nepal</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -7234,29 +7234,29 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Kathmandu</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>NP</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>KJA</t>
+          <t>CCU</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Krasnoyarsk, Russia</t>
+          <t>Kolkata, India</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -7266,29 +7266,29 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Krasnoyarsk</t>
+          <t>Kolkata</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>KUL</t>
+          <t>KJA</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>Krasnoyarsk, Russia</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -7298,29 +7298,29 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Kuala Lumpur</t>
+          <t>Krasnoyarsk</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>RU</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>PKX</t>
+          <t>KUL</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Langfang, China</t>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -7330,29 +7330,29 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Langfang</t>
+          <t>Kuala Lumpur</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>MFM</t>
+          <t>PKX</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Macau</t>
+          <t>Langfang, China</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -7360,19 +7360,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr"/>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Langfang</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>MLE</t>
+          <t>MFM</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Malé, Maldives</t>
+          <t>Macau</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -7380,31 +7392,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>Malé</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>Maldives</t>
-        </is>
-      </c>
-      <c r="F220" t="inlineStr">
-        <is>
-          <t>MV</t>
-        </is>
-      </c>
+      <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>MNL</t>
+          <t>MLE</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Manila, Philippines</t>
+          <t>Malé, Maldives</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -7414,29 +7414,29 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Manila</t>
+          <t>Malé</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Maldives</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>MV</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>MNL</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>Manila, Philippines</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -7446,29 +7446,29 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>NAG</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Nagpur, India</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -7495,12 +7495,12 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>OKA</t>
+          <t>NAG</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Naha, Japan</t>
+          <t>Nagpur, India</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -7510,29 +7510,29 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Naha</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>DEL</t>
+          <t>OKA</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>New Delhi, India</t>
+          <t>Naha, Japan</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -7542,29 +7542,29 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Naha</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>KIX</t>
+          <t>DEL</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Osaka, Japan</t>
+          <t>New Delhi, India</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -7574,29 +7574,29 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Osaka</t>
+          <t>New Delhi</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>PAT</t>
+          <t>KIX</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Patna, India</t>
+          <t>Osaka, Japan</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -7606,29 +7606,29 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Patna</t>
+          <t>Osaka</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>PNH</t>
+          <t>PAT</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Phnom Penh, Cambodia</t>
+          <t>Patna, India</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -7638,29 +7638,29 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Phnom Penh</t>
+          <t>Patna</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>KH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>PNH</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Qingdao, China</t>
+          <t>Phnom Penh, Cambodia</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -7670,29 +7670,29 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Qingdao</t>
+          <t>Phnom Penh</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KH</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>ICN</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Qingdao, China</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -7702,29 +7702,29 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Qingdao</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>ICN</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Shanghai, China</t>
+          <t>Seoul, South Korea</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -7734,29 +7734,29 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Shanghai</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KR</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Singapore, Singapore</t>
+          <t>Shanghai, China</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -7766,29 +7766,29 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Shanghai</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>URT</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Surat Thani, Thailand</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -7798,29 +7798,29 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Surat Thani</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>SG</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>URT</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Surat Thani, Thailand</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -7828,19 +7828,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr"/>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Surat Thani</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>NRT</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -7848,31 +7860,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>Tokyo</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="F235" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>ULN</t>
+          <t>NRT</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Ulaanbaatar, Mongolia</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -7882,29 +7882,29 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Ulaanbaatar</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Mongolia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>VTE</t>
+          <t>ULN</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Vientiane, Laos</t>
+          <t>Ulaanbaatar, Mongolia</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -7914,29 +7914,29 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Vientiane</t>
+          <t>Ulaanbaatar</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Laos</t>
+          <t>Mongolia</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>MN</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>KHN</t>
+          <t>VTE</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Xinyu, China</t>
+          <t>Vientiane, Laos</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -7946,29 +7946,29 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Xinyu</t>
+          <t>Vientiane</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Laos</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>LA</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>EVN</t>
+          <t>KHN</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Yerevan, Armenia</t>
+          <t>Xinyu, China</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -7978,29 +7978,29 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Yerevan</t>
+          <t>Xinyu</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Armenia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>JOG</t>
+          <t>EVN</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Yogyakarta, Indonesia</t>
+          <t>Yerevan, Armenia</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -8010,29 +8010,29 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Yogyakarta</t>
+          <t>Yerevan</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Armenia</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>AM</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>JOG</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Cagayan de Oro, Philippines</t>
+          <t>Yogyakarta, Indonesia</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -8042,29 +8042,29 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Cagayan de Oro</t>
+          <t>Yogyakarta</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>COK</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Kochi, India</t>
+          <t>Cagayan de Oro, Philippines</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -8074,29 +8074,29 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Cagayan de Oro</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>COK</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Denpasar, Indonesia</t>
+          <t>Kochi, India</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -8106,29 +8106,29 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Denpasar</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>CNN</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Kannur, India</t>
+          <t>Denpasar, Indonesia</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -8138,29 +8138,29 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Kannur</t>
+          <t>Denpasar</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>SZX</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Shenzhen, China</t>
+          <t>Kannur, India</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -8170,29 +8170,29 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Shenzhen</t>
+          <t>Kannur</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>KWE</t>
+          <t>SZX</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Guiyang, China</t>
+          <t>Shenzhen, China</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Guiyang</t>
+          <t>Shenzhen</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -8219,12 +8219,12 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>HGH</t>
+          <t>KWE</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Shaoxing, China</t>
+          <t>Guiyang, China</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Shaoxing</t>
+          <t>Guiyang</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -8251,12 +8251,12 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>CZX</t>
+          <t>HGH</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Changzhou, China</t>
+          <t>Shaoxing, China</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Changzhou</t>
+          <t>Shaoxing</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -8283,12 +8283,12 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>KMG</t>
+          <t>CZX</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Kunming, China</t>
+          <t>Changzhou, China</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Kunming</t>
+          <t>Changzhou</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -8315,12 +8315,12 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>CNX</t>
+          <t>KMG</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Chiang Mai, Thailand</t>
+          <t>Kunming, China</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -8330,29 +8330,29 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Chiang Mai</t>
+          <t>Kunming</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>CGO</t>
+          <t>CNX</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Zhengzhou, China</t>
+          <t>Chiang Mai, Thailand</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -8362,29 +8362,29 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Zhengzhou</t>
+          <t>Chiang Mai</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>TYN</t>
+          <t>CGO</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Yangquan, China</t>
+          <t>Zhengzhou, China</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Yangquan</t>
+          <t>Zhengzhou</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -8411,12 +8411,12 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>TYN</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Changsha, China</t>
+          <t>Yangquan, China</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Changsha</t>
+          <t>Yangquan</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -8443,12 +8443,12 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>DLC</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Dalian, China</t>
+          <t>Changsha, China</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Dalian</t>
+          <t>Changsha</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -8475,12 +8475,12 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>BHY</t>
+          <t>DLC</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Beihai, China</t>
+          <t>Dalian, China</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Beihai</t>
+          <t>Dalian</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -8507,12 +8507,12 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>CKG</t>
+          <t>BHY</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Chongqing, China</t>
+          <t>Beihai, China</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Chongqing</t>
+          <t>Beihai</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -8539,12 +8539,12 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>XFN</t>
+          <t>CKG</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Xiangyang, China</t>
+          <t>Chongqing, China</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Xiangyang</t>
+          <t>Chongqing</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -8571,12 +8571,12 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>DAD</t>
+          <t>XFN</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Da Nang, Vietnam</t>
+          <t>Xiangyang, China</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -8586,29 +8586,29 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Xiangyang</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>JXG</t>
+          <t>DAD</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Jiaxing, China</t>
+          <t>Da Nang, Vietnam</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -8618,29 +8618,29 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Jiaxing</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>CRK</t>
+          <t>JXG</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Tarlac City, Philippines</t>
+          <t>Jiaxing, China</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -8650,29 +8650,29 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Tarlac City</t>
+          <t>Jiaxing</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>PBH</t>
+          <t>CRK</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Thimphu, Bhutan</t>
+          <t>Tarlac City, Philippines</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -8682,29 +8682,29 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Thimphu</t>
+          <t>Tarlac City</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>BT</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>XIY</t>
+          <t>PBH</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Baoji, China</t>
+          <t>Thimphu, Bhutan</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -8714,29 +8714,29 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Baoji</t>
+          <t>Thimphu</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>BT</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>NQZ</t>
+          <t>XIY</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Astana, Kazakhstan</t>
+          <t>Baoji, China</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -8746,29 +8746,29 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Astana</t>
+          <t>Baoji</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>NQZ</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -8778,29 +8778,29 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Astana</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -8810,29 +8810,29 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Aktobe</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -8842,29 +8842,29 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Aktobe</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -8891,12 +8891,12 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -8906,29 +8906,29 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -8938,29 +8938,29 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Malang</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>KG</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -8970,29 +8970,29 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Malang</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -9002,29 +9002,29 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Chengdu</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -9034,29 +9034,29 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Agra</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -9066,7 +9066,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Agra</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -9083,12 +9083,12 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -9098,29 +9098,29 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Coimbatore</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -9130,29 +9130,29 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -9162,29 +9162,29 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -9194,29 +9194,29 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9226,7 +9226,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Sambalpur</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -9243,44 +9243,44 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Sambalpur</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9307,12 +9307,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9339,12 +9339,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9371,12 +9371,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9403,12 +9403,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,29 +9514,29 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,29 +9546,29 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9595,12 +9595,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9627,12 +9627,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,29 +9802,29 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,29 +9834,29 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,29 +9866,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9915,12 +9915,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9947,12 +9947,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,7 +9994,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10011,12 +10011,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,29 +10026,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,29 +10058,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,29 +10154,29 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,29 +10186,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,7 +10218,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10235,12 +10235,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,29 +10282,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10331,12 +10331,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10363,12 +10363,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,29 +10570,29 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,29 +10602,29 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,29 +10826,29 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,29 +10858,29 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,29 +11018,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,30 +11099,62 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B338" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C338" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D338" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E338" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F338" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>